<commit_message>
Normalize Fast Forward (ZzZ / Timelapse) combat delays to match Natural play
Previously, `runFastForward()` ignored game UI delays, such as sliding animations (1000ms), visual fainting (500ms), and stat-based attack delays. This caused offline and timelapse modes to farm ~2.6x faster than natural play.

This commit updates the fast-forward combat time accumulator to simulate these missing UI delays, ensuring offline progression perfectly matches active play.

It also includes the generated .xlsx and .md reports analyzing these changes.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Hunting_Analysis_Report.xlsx
+++ b/Hunting_Analysis_Report.xlsx
@@ -511,22 +511,22 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>2400</v>
+        <v>900</v>
       </c>
       <c r="D5">
-        <v>2280</v>
+        <v>855</v>
       </c>
       <c r="E5">
-        <v>12000</v>
+        <v>4500</v>
       </c>
       <c r="F5">
-        <v>60000</v>
+        <v>22500</v>
       </c>
       <c r="G5">
-        <v>1500</v>
+        <v>4000</v>
       </c>
       <c r="H5" t="str">
-        <v>Static calculation. Not affected by game speed.</v>
+        <v>Scales linearly. Combines Search, Slide, Attack and Defeat Delays.</v>
       </c>
     </row>
     <row r="6">
@@ -537,22 +537,22 @@
         <v>1</v>
       </c>
       <c r="C6">
-        <v>2400</v>
+        <v>900</v>
       </c>
       <c r="D6">
-        <v>2280</v>
+        <v>855</v>
       </c>
       <c r="E6">
-        <v>12000</v>
+        <v>4500</v>
       </c>
       <c r="F6">
-        <v>60000</v>
+        <v>22500</v>
       </c>
       <c r="G6">
-        <v>1500</v>
+        <v>4000</v>
       </c>
       <c r="H6" t="str">
-        <v>Static calculation. Not affected by game speed.</v>
+        <v>Scales linearly. Combines Search, Slide, Attack and Defeat Delays.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>